<commit_message>
update: redesain panel & data preparatio, fix bug
</commit_message>
<xml_diff>
--- a/assets/Template Format Individu.xlsx
+++ b/assets/Template Format Individu.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yazj8\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Downloads\ckg-auto-chrome-extensions-main\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6B066081-2377-432D-8F2A-43325C0A76B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76B99BBC-49BD-495E-9890-2B681CF13173}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="4" r:id="rId1"/>
@@ -83,6 +83,17 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext uri="GoogleSheetsCustomDataVersion2">
       <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId9" roundtripDataChecksum="cIhN11uw6wPbmyeQUk1+2uXeZYsK6xilcwTck8tAqYY="/>
     </ext>
@@ -1010,50 +1021,50 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:CP151"/>
-  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="21.6" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="21.6" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.6640625" customWidth="1"/>
-    <col min="2" max="2" width="22.5546875" customWidth="1"/>
+    <col min="1" max="1" width="8.7109375" customWidth="1"/>
+    <col min="2" max="2" width="22.5703125" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
-    <col min="4" max="4" width="19.33203125" customWidth="1"/>
-    <col min="5" max="5" width="18.33203125" customWidth="1"/>
+    <col min="4" max="4" width="19.28515625" customWidth="1"/>
+    <col min="5" max="5" width="18.28515625" customWidth="1"/>
     <col min="6" max="6" width="21" customWidth="1"/>
-    <col min="7" max="7" width="33.33203125" customWidth="1"/>
-    <col min="8" max="8" width="18.109375" customWidth="1"/>
-    <col min="9" max="9" width="29.88671875" customWidth="1"/>
+    <col min="7" max="7" width="33.28515625" customWidth="1"/>
+    <col min="8" max="8" width="18.140625" customWidth="1"/>
+    <col min="9" max="9" width="29.85546875" customWidth="1"/>
     <col min="10" max="10" width="28" customWidth="1"/>
     <col min="11" max="11" width="26" customWidth="1"/>
-    <col min="12" max="12" width="32.5546875" customWidth="1"/>
-    <col min="13" max="13" width="50.109375" customWidth="1"/>
+    <col min="12" max="12" width="32.5703125" customWidth="1"/>
+    <col min="13" max="13" width="50.140625" customWidth="1"/>
     <col min="14" max="27" width="28" customWidth="1"/>
-    <col min="28" max="34" width="18.109375" customWidth="1"/>
-    <col min="35" max="41" width="12.88671875" customWidth="1"/>
-    <col min="42" max="44" width="31.88671875" customWidth="1"/>
-    <col min="45" max="45" width="29.44140625" customWidth="1"/>
-    <col min="46" max="46" width="30.109375" customWidth="1"/>
-    <col min="47" max="65" width="25.5546875" customWidth="1"/>
-    <col min="66" max="69" width="22.88671875" customWidth="1"/>
-    <col min="70" max="70" width="20.109375" customWidth="1"/>
+    <col min="28" max="34" width="18.140625" customWidth="1"/>
+    <col min="35" max="41" width="12.85546875" customWidth="1"/>
+    <col min="42" max="44" width="31.85546875" customWidth="1"/>
+    <col min="45" max="45" width="29.42578125" customWidth="1"/>
+    <col min="46" max="46" width="30.140625" customWidth="1"/>
+    <col min="47" max="65" width="25.5703125" customWidth="1"/>
+    <col min="66" max="69" width="22.85546875" customWidth="1"/>
+    <col min="70" max="70" width="20.140625" customWidth="1"/>
     <col min="71" max="71" width="35" customWidth="1"/>
-    <col min="72" max="72" width="27.109375" customWidth="1"/>
+    <col min="72" max="72" width="27.140625" customWidth="1"/>
     <col min="73" max="73" width="22" customWidth="1"/>
-    <col min="74" max="74" width="27.44140625" customWidth="1"/>
-    <col min="75" max="75" width="11.33203125" customWidth="1"/>
-    <col min="76" max="76" width="15.88671875" customWidth="1"/>
-    <col min="77" max="77" width="8.6640625" customWidth="1"/>
-    <col min="78" max="78" width="19.5546875" customWidth="1"/>
+    <col min="74" max="74" width="27.42578125" customWidth="1"/>
+    <col min="75" max="75" width="11.28515625" customWidth="1"/>
+    <col min="76" max="76" width="15.85546875" customWidth="1"/>
+    <col min="77" max="77" width="8.7109375" customWidth="1"/>
+    <col min="78" max="78" width="19.5703125" customWidth="1"/>
     <col min="79" max="79" width="21" customWidth="1"/>
     <col min="80" max="80" width="22" customWidth="1"/>
-    <col min="81" max="81" width="23.109375" customWidth="1"/>
-    <col min="82" max="82" width="24.33203125" customWidth="1"/>
-    <col min="83" max="89" width="13.33203125" customWidth="1"/>
-    <col min="90" max="90" width="20.33203125" customWidth="1"/>
-    <col min="91" max="92" width="8.6640625" customWidth="1"/>
-    <col min="93" max="93" width="18.6640625" customWidth="1"/>
+    <col min="81" max="81" width="23.140625" customWidth="1"/>
+    <col min="82" max="82" width="24.28515625" customWidth="1"/>
+    <col min="83" max="89" width="13.28515625" customWidth="1"/>
+    <col min="90" max="90" width="20.28515625" customWidth="1"/>
+    <col min="91" max="92" width="8.7109375" customWidth="1"/>
+    <col min="93" max="93" width="18.7109375" customWidth="1"/>
     <col min="94" max="94" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:94" s="1" customFormat="1" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:94" s="1" customFormat="1" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
@@ -1337,7 +1348,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="2" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="5">
         <v>1</v>
       </c>
@@ -1587,14 +1598,14 @@
         <v>OBESITAS</v>
       </c>
     </row>
-    <row r="3" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5"/>
       <c r="B3" s="15"/>
       <c r="C3" s="14"/>
       <c r="D3" s="6"/>
       <c r="E3" s="14"/>
       <c r="F3" s="25"/>
-      <c r="G3" s="24"/>
+      <c r="G3" s="23"/>
       <c r="H3" s="29"/>
       <c r="I3" s="27"/>
       <c r="J3" s="5"/>
@@ -1683,7 +1694,7 @@
       <c r="CO3" s="14"/>
       <c r="CP3" s="14"/>
     </row>
-    <row r="4" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5"/>
       <c r="B4" s="15"/>
       <c r="C4" s="14"/>
@@ -1779,7 +1790,7 @@
       <c r="CO4" s="14"/>
       <c r="CP4" s="14"/>
     </row>
-    <row r="5" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5"/>
       <c r="B5" s="15"/>
       <c r="C5" s="14"/>
@@ -1875,7 +1886,7 @@
       <c r="CO5" s="14"/>
       <c r="CP5" s="14"/>
     </row>
-    <row r="6" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5"/>
       <c r="B6" s="15"/>
       <c r="C6" s="14"/>
@@ -1971,7 +1982,7 @@
       <c r="CO6" s="14"/>
       <c r="CP6" s="14"/>
     </row>
-    <row r="7" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5"/>
       <c r="B7" s="15"/>
       <c r="C7" s="14"/>
@@ -2067,7 +2078,7 @@
       <c r="CO7" s="14"/>
       <c r="CP7" s="14"/>
     </row>
-    <row r="8" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5"/>
       <c r="B8" s="15"/>
       <c r="C8" s="14"/>
@@ -2163,7 +2174,7 @@
       <c r="CO8" s="14"/>
       <c r="CP8" s="14"/>
     </row>
-    <row r="9" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5"/>
       <c r="B9" s="15"/>
       <c r="C9" s="14"/>
@@ -2259,7 +2270,7 @@
       <c r="CO9" s="14"/>
       <c r="CP9" s="14"/>
     </row>
-    <row r="10" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5"/>
       <c r="B10" s="15"/>
       <c r="C10" s="14"/>
@@ -2355,7 +2366,7 @@
       <c r="CO10" s="14"/>
       <c r="CP10" s="14"/>
     </row>
-    <row r="11" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5"/>
       <c r="B11" s="15"/>
       <c r="C11" s="14"/>
@@ -2451,7 +2462,7 @@
       <c r="CO11" s="14"/>
       <c r="CP11" s="14"/>
     </row>
-    <row r="12" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="5"/>
       <c r="B12" s="15"/>
       <c r="C12" s="14"/>
@@ -2547,7 +2558,7 @@
       <c r="CO12" s="14"/>
       <c r="CP12" s="14"/>
     </row>
-    <row r="13" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="5"/>
       <c r="B13" s="15"/>
       <c r="C13" s="14"/>
@@ -2643,7 +2654,7 @@
       <c r="CO13" s="14"/>
       <c r="CP13" s="14"/>
     </row>
-    <row r="14" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="5"/>
       <c r="B14" s="15"/>
       <c r="C14" s="14"/>
@@ -2739,7 +2750,7 @@
       <c r="CO14" s="14"/>
       <c r="CP14" s="14"/>
     </row>
-    <row r="15" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="5"/>
       <c r="B15" s="15"/>
       <c r="C15" s="14"/>
@@ -2835,7 +2846,7 @@
       <c r="CO15" s="14"/>
       <c r="CP15" s="14"/>
     </row>
-    <row r="16" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="5"/>
       <c r="B16" s="15"/>
       <c r="C16" s="14"/>
@@ -2931,7 +2942,7 @@
       <c r="CO16" s="14"/>
       <c r="CP16" s="14"/>
     </row>
-    <row r="17" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="5"/>
       <c r="B17" s="15"/>
       <c r="C17" s="14"/>
@@ -3027,7 +3038,7 @@
       <c r="CO17" s="14"/>
       <c r="CP17" s="14"/>
     </row>
-    <row r="18" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="5"/>
       <c r="B18" s="15"/>
       <c r="C18" s="14"/>
@@ -3123,7 +3134,7 @@
       <c r="CO18" s="14"/>
       <c r="CP18" s="14"/>
     </row>
-    <row r="19" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="5"/>
       <c r="B19" s="15"/>
       <c r="C19" s="14"/>
@@ -3219,7 +3230,7 @@
       <c r="CO19" s="14"/>
       <c r="CP19" s="14"/>
     </row>
-    <row r="20" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="5"/>
       <c r="B20" s="15"/>
       <c r="C20" s="14"/>
@@ -3315,7 +3326,7 @@
       <c r="CO20" s="14"/>
       <c r="CP20" s="14"/>
     </row>
-    <row r="21" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="5"/>
       <c r="B21" s="15"/>
       <c r="C21" s="14"/>
@@ -3411,7 +3422,7 @@
       <c r="CO21" s="14"/>
       <c r="CP21" s="14"/>
     </row>
-    <row r="22" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="5"/>
       <c r="B22" s="15"/>
       <c r="C22" s="14"/>
@@ -3507,7 +3518,7 @@
       <c r="CO22" s="14"/>
       <c r="CP22" s="14"/>
     </row>
-    <row r="23" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="5"/>
       <c r="B23" s="15"/>
       <c r="C23" s="14"/>
@@ -3603,7 +3614,7 @@
       <c r="CO23" s="14"/>
       <c r="CP23" s="14"/>
     </row>
-    <row r="24" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="5"/>
       <c r="B24" s="15"/>
       <c r="C24" s="14"/>
@@ -3699,7 +3710,7 @@
       <c r="CO24" s="14"/>
       <c r="CP24" s="14"/>
     </row>
-    <row r="25" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="5"/>
       <c r="B25" s="15"/>
       <c r="C25" s="14"/>
@@ -3795,7 +3806,7 @@
       <c r="CO25" s="14"/>
       <c r="CP25" s="14"/>
     </row>
-    <row r="26" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="5"/>
       <c r="B26" s="15"/>
       <c r="C26" s="14"/>
@@ -3891,7 +3902,7 @@
       <c r="CO26" s="14"/>
       <c r="CP26" s="14"/>
     </row>
-    <row r="27" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="5"/>
       <c r="B27" s="15"/>
       <c r="C27" s="14"/>
@@ -3987,7 +3998,7 @@
       <c r="CO27" s="14"/>
       <c r="CP27" s="14"/>
     </row>
-    <row r="28" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="5"/>
       <c r="B28" s="15"/>
       <c r="C28" s="14"/>
@@ -4083,7 +4094,7 @@
       <c r="CO28" s="14"/>
       <c r="CP28" s="14"/>
     </row>
-    <row r="29" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="5"/>
       <c r="B29" s="15"/>
       <c r="C29" s="14"/>
@@ -4179,7 +4190,7 @@
       <c r="CO29" s="14"/>
       <c r="CP29" s="14"/>
     </row>
-    <row r="30" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="5"/>
       <c r="B30" s="15"/>
       <c r="C30" s="14"/>
@@ -4275,7 +4286,7 @@
       <c r="CO30" s="14"/>
       <c r="CP30" s="14"/>
     </row>
-    <row r="31" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="5"/>
       <c r="B31" s="15"/>
       <c r="C31" s="14"/>
@@ -4371,7 +4382,7 @@
       <c r="CO31" s="14"/>
       <c r="CP31" s="14"/>
     </row>
-    <row r="32" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="5"/>
       <c r="B32" s="15"/>
       <c r="C32" s="14"/>
@@ -4467,7 +4478,7 @@
       <c r="CO32" s="14"/>
       <c r="CP32" s="14"/>
     </row>
-    <row r="33" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="5"/>
       <c r="B33" s="15"/>
       <c r="C33" s="14"/>
@@ -4563,7 +4574,7 @@
       <c r="CO33" s="14"/>
       <c r="CP33" s="14"/>
     </row>
-    <row r="34" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="5"/>
       <c r="B34" s="15"/>
       <c r="C34" s="14"/>
@@ -4659,7 +4670,7 @@
       <c r="CO34" s="14"/>
       <c r="CP34" s="14"/>
     </row>
-    <row r="35" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="5"/>
       <c r="B35" s="15"/>
       <c r="C35" s="14"/>
@@ -4755,7 +4766,7 @@
       <c r="CO35" s="14"/>
       <c r="CP35" s="14"/>
     </row>
-    <row r="36" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="5"/>
       <c r="B36" s="15"/>
       <c r="C36" s="14"/>
@@ -4851,7 +4862,7 @@
       <c r="CO36" s="14"/>
       <c r="CP36" s="14"/>
     </row>
-    <row r="37" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="5"/>
       <c r="B37" s="15"/>
       <c r="C37" s="14"/>
@@ -4947,7 +4958,7 @@
       <c r="CO37" s="14"/>
       <c r="CP37" s="14"/>
     </row>
-    <row r="38" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="5"/>
       <c r="B38" s="15"/>
       <c r="C38" s="14"/>
@@ -5043,7 +5054,7 @@
       <c r="CO38" s="14"/>
       <c r="CP38" s="14"/>
     </row>
-    <row r="39" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="5"/>
       <c r="B39" s="15"/>
       <c r="C39" s="14"/>
@@ -5139,7 +5150,7 @@
       <c r="CO39" s="14"/>
       <c r="CP39" s="14"/>
     </row>
-    <row r="40" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="5"/>
       <c r="B40" s="15"/>
       <c r="C40" s="14"/>
@@ -5235,7 +5246,7 @@
       <c r="CO40" s="14"/>
       <c r="CP40" s="14"/>
     </row>
-    <row r="41" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="5"/>
       <c r="B41" s="15"/>
       <c r="C41" s="14"/>
@@ -5331,7 +5342,7 @@
       <c r="CO41" s="14"/>
       <c r="CP41" s="14"/>
     </row>
-    <row r="42" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="5"/>
       <c r="B42" s="15"/>
       <c r="C42" s="14"/>
@@ -5427,7 +5438,7 @@
       <c r="CO42" s="14"/>
       <c r="CP42" s="14"/>
     </row>
-    <row r="43" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="5"/>
       <c r="B43" s="15"/>
       <c r="C43" s="14"/>
@@ -5523,7 +5534,7 @@
       <c r="CO43" s="14"/>
       <c r="CP43" s="14"/>
     </row>
-    <row r="44" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="5"/>
       <c r="B44" s="15"/>
       <c r="C44" s="14"/>
@@ -5619,7 +5630,7 @@
       <c r="CO44" s="14"/>
       <c r="CP44" s="14"/>
     </row>
-    <row r="45" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="5"/>
       <c r="B45" s="15"/>
       <c r="C45" s="14"/>
@@ -5715,7 +5726,7 @@
       <c r="CO45" s="14"/>
       <c r="CP45" s="14"/>
     </row>
-    <row r="46" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="5"/>
       <c r="B46" s="15"/>
       <c r="C46" s="14"/>
@@ -5811,7 +5822,7 @@
       <c r="CO46" s="14"/>
       <c r="CP46" s="14"/>
     </row>
-    <row r="47" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="5"/>
       <c r="B47" s="15"/>
       <c r="C47" s="14"/>
@@ -5907,7 +5918,7 @@
       <c r="CO47" s="14"/>
       <c r="CP47" s="14"/>
     </row>
-    <row r="48" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="5"/>
       <c r="B48" s="15"/>
       <c r="C48" s="14"/>
@@ -6003,7 +6014,7 @@
       <c r="CO48" s="14"/>
       <c r="CP48" s="14"/>
     </row>
-    <row r="49" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" s="5"/>
       <c r="B49" s="15"/>
       <c r="C49" s="14"/>
@@ -6099,7 +6110,7 @@
       <c r="CO49" s="14"/>
       <c r="CP49" s="14"/>
     </row>
-    <row r="50" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="5"/>
       <c r="B50" s="15"/>
       <c r="C50" s="14"/>
@@ -6195,7 +6206,7 @@
       <c r="CO50" s="14"/>
       <c r="CP50" s="14"/>
     </row>
-    <row r="51" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="5"/>
       <c r="B51" s="15"/>
       <c r="C51" s="14"/>
@@ -6291,7 +6302,7 @@
       <c r="CO51" s="14"/>
       <c r="CP51" s="14"/>
     </row>
-    <row r="52" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="5"/>
       <c r="B52" s="15"/>
       <c r="C52" s="14"/>
@@ -6387,7 +6398,7 @@
       <c r="CO52" s="14"/>
       <c r="CP52" s="14"/>
     </row>
-    <row r="53" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="5"/>
       <c r="B53" s="15"/>
       <c r="C53" s="14"/>
@@ -6483,7 +6494,7 @@
       <c r="CO53" s="14"/>
       <c r="CP53" s="14"/>
     </row>
-    <row r="54" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="5"/>
       <c r="B54" s="15"/>
       <c r="C54" s="14"/>
@@ -6579,7 +6590,7 @@
       <c r="CO54" s="14"/>
       <c r="CP54" s="14"/>
     </row>
-    <row r="55" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A55" s="5"/>
       <c r="B55" s="15"/>
       <c r="C55" s="14"/>
@@ -6675,7 +6686,7 @@
       <c r="CO55" s="14"/>
       <c r="CP55" s="14"/>
     </row>
-    <row r="56" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="5"/>
       <c r="B56" s="15"/>
       <c r="C56" s="14"/>
@@ -6771,7 +6782,7 @@
       <c r="CO56" s="14"/>
       <c r="CP56" s="14"/>
     </row>
-    <row r="57" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57" s="5"/>
       <c r="B57" s="15"/>
       <c r="C57" s="14"/>
@@ -6867,7 +6878,7 @@
       <c r="CO57" s="14"/>
       <c r="CP57" s="14"/>
     </row>
-    <row r="58" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A58" s="5"/>
       <c r="B58" s="15"/>
       <c r="C58" s="14"/>
@@ -6963,7 +6974,7 @@
       <c r="CO58" s="14"/>
       <c r="CP58" s="14"/>
     </row>
-    <row r="59" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="5"/>
       <c r="B59" s="15"/>
       <c r="C59" s="14"/>
@@ -7059,7 +7070,7 @@
       <c r="CO59" s="14"/>
       <c r="CP59" s="14"/>
     </row>
-    <row r="60" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A60" s="5"/>
       <c r="B60" s="15"/>
       <c r="C60" s="14"/>
@@ -7155,7 +7166,7 @@
       <c r="CO60" s="14"/>
       <c r="CP60" s="14"/>
     </row>
-    <row r="61" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A61" s="5"/>
       <c r="B61" s="15"/>
       <c r="C61" s="14"/>
@@ -7251,7 +7262,7 @@
       <c r="CO61" s="14"/>
       <c r="CP61" s="14"/>
     </row>
-    <row r="62" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A62" s="5"/>
       <c r="B62" s="15"/>
       <c r="C62" s="14"/>
@@ -7347,7 +7358,7 @@
       <c r="CO62" s="14"/>
       <c r="CP62" s="14"/>
     </row>
-    <row r="63" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A63" s="5"/>
       <c r="B63" s="15"/>
       <c r="C63" s="14"/>
@@ -7443,7 +7454,7 @@
       <c r="CO63" s="14"/>
       <c r="CP63" s="14"/>
     </row>
-    <row r="64" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A64" s="5"/>
       <c r="B64" s="15"/>
       <c r="C64" s="14"/>
@@ -7539,7 +7550,7 @@
       <c r="CO64" s="14"/>
       <c r="CP64" s="14"/>
     </row>
-    <row r="65" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A65" s="5"/>
       <c r="B65" s="15"/>
       <c r="C65" s="14"/>
@@ -7635,7 +7646,7 @@
       <c r="CO65" s="14"/>
       <c r="CP65" s="14"/>
     </row>
-    <row r="66" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="5"/>
       <c r="B66" s="15"/>
       <c r="C66" s="14"/>
@@ -7731,7 +7742,7 @@
       <c r="CO66" s="14"/>
       <c r="CP66" s="14"/>
     </row>
-    <row r="67" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A67" s="5"/>
       <c r="B67" s="15"/>
       <c r="C67" s="14"/>
@@ -7827,7 +7838,7 @@
       <c r="CO67" s="14"/>
       <c r="CP67" s="14"/>
     </row>
-    <row r="68" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A68" s="5"/>
       <c r="B68" s="15"/>
       <c r="C68" s="14"/>
@@ -7923,7 +7934,7 @@
       <c r="CO68" s="14"/>
       <c r="CP68" s="14"/>
     </row>
-    <row r="69" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A69" s="5"/>
       <c r="B69" s="15"/>
       <c r="C69" s="14"/>
@@ -8019,7 +8030,7 @@
       <c r="CO69" s="14"/>
       <c r="CP69" s="14"/>
     </row>
-    <row r="70" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A70" s="5"/>
       <c r="B70" s="15"/>
       <c r="C70" s="14"/>
@@ -8115,7 +8126,7 @@
       <c r="CO70" s="14"/>
       <c r="CP70" s="14"/>
     </row>
-    <row r="71" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A71" s="5"/>
       <c r="B71" s="15"/>
       <c r="C71" s="14"/>
@@ -8211,7 +8222,7 @@
       <c r="CO71" s="14"/>
       <c r="CP71" s="14"/>
     </row>
-    <row r="72" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A72" s="5"/>
       <c r="B72" s="15"/>
       <c r="C72" s="14"/>
@@ -8307,7 +8318,7 @@
       <c r="CO72" s="14"/>
       <c r="CP72" s="14"/>
     </row>
-    <row r="73" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A73" s="5"/>
       <c r="B73" s="15"/>
       <c r="C73" s="14"/>
@@ -8403,7 +8414,7 @@
       <c r="CO73" s="14"/>
       <c r="CP73" s="14"/>
     </row>
-    <row r="74" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A74" s="5"/>
       <c r="B74" s="15"/>
       <c r="C74" s="14"/>
@@ -8499,7 +8510,7 @@
       <c r="CO74" s="14"/>
       <c r="CP74" s="14"/>
     </row>
-    <row r="75" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A75" s="5"/>
       <c r="B75" s="15"/>
       <c r="C75" s="14"/>
@@ -8595,7 +8606,7 @@
       <c r="CO75" s="14"/>
       <c r="CP75" s="14"/>
     </row>
-    <row r="76" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A76" s="5"/>
       <c r="B76" s="15"/>
       <c r="C76" s="14"/>
@@ -8691,7 +8702,7 @@
       <c r="CO76" s="14"/>
       <c r="CP76" s="14"/>
     </row>
-    <row r="77" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A77" s="5"/>
       <c r="B77" s="15"/>
       <c r="C77" s="14"/>
@@ -8787,7 +8798,7 @@
       <c r="CO77" s="14"/>
       <c r="CP77" s="14"/>
     </row>
-    <row r="78" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A78" s="5"/>
       <c r="B78" s="15"/>
       <c r="C78" s="14"/>
@@ -8883,7 +8894,7 @@
       <c r="CO78" s="14"/>
       <c r="CP78" s="14"/>
     </row>
-    <row r="79" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A79" s="5"/>
       <c r="B79" s="15"/>
       <c r="C79" s="14"/>
@@ -8979,7 +8990,7 @@
       <c r="CO79" s="14"/>
       <c r="CP79" s="14"/>
     </row>
-    <row r="80" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A80" s="5"/>
       <c r="B80" s="15"/>
       <c r="C80" s="14"/>
@@ -9075,7 +9086,7 @@
       <c r="CO80" s="14"/>
       <c r="CP80" s="14"/>
     </row>
-    <row r="81" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A81" s="5"/>
       <c r="B81" s="15"/>
       <c r="C81" s="14"/>
@@ -9171,7 +9182,7 @@
       <c r="CO81" s="14"/>
       <c r="CP81" s="14"/>
     </row>
-    <row r="82" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A82" s="5"/>
       <c r="B82" s="15"/>
       <c r="C82" s="14"/>
@@ -9267,7 +9278,7 @@
       <c r="CO82" s="14"/>
       <c r="CP82" s="14"/>
     </row>
-    <row r="83" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A83" s="5"/>
       <c r="B83" s="15"/>
       <c r="C83" s="14"/>
@@ -9363,7 +9374,7 @@
       <c r="CO83" s="14"/>
       <c r="CP83" s="14"/>
     </row>
-    <row r="84" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A84" s="5"/>
       <c r="B84" s="15"/>
       <c r="C84" s="14"/>
@@ -9459,7 +9470,7 @@
       <c r="CO84" s="14"/>
       <c r="CP84" s="14"/>
     </row>
-    <row r="85" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A85" s="5"/>
       <c r="B85" s="15"/>
       <c r="C85" s="14"/>
@@ -9555,7 +9566,7 @@
       <c r="CO85" s="14"/>
       <c r="CP85" s="14"/>
     </row>
-    <row r="86" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A86" s="5"/>
       <c r="B86" s="15"/>
       <c r="C86" s="14"/>
@@ -9651,7 +9662,7 @@
       <c r="CO86" s="14"/>
       <c r="CP86" s="14"/>
     </row>
-    <row r="87" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A87" s="5"/>
       <c r="B87" s="15"/>
       <c r="C87" s="14"/>
@@ -9747,7 +9758,7 @@
       <c r="CO87" s="14"/>
       <c r="CP87" s="14"/>
     </row>
-    <row r="88" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A88" s="5"/>
       <c r="B88" s="15"/>
       <c r="C88" s="14"/>
@@ -9843,7 +9854,7 @@
       <c r="CO88" s="14"/>
       <c r="CP88" s="14"/>
     </row>
-    <row r="89" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A89" s="5"/>
       <c r="B89" s="15"/>
       <c r="C89" s="14"/>
@@ -9939,7 +9950,7 @@
       <c r="CO89" s="14"/>
       <c r="CP89" s="14"/>
     </row>
-    <row r="90" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A90" s="5"/>
       <c r="B90" s="15"/>
       <c r="C90" s="14"/>
@@ -10035,7 +10046,7 @@
       <c r="CO90" s="14"/>
       <c r="CP90" s="14"/>
     </row>
-    <row r="91" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A91" s="5"/>
       <c r="B91" s="15"/>
       <c r="C91" s="14"/>
@@ -10131,7 +10142,7 @@
       <c r="CO91" s="14"/>
       <c r="CP91" s="14"/>
     </row>
-    <row r="92" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A92" s="5"/>
       <c r="B92" s="15"/>
       <c r="C92" s="14"/>
@@ -10227,7 +10238,7 @@
       <c r="CO92" s="14"/>
       <c r="CP92" s="14"/>
     </row>
-    <row r="93" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A93" s="5"/>
       <c r="B93" s="15"/>
       <c r="C93" s="14"/>
@@ -10323,7 +10334,7 @@
       <c r="CO93" s="14"/>
       <c r="CP93" s="14"/>
     </row>
-    <row r="94" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A94" s="5"/>
       <c r="B94" s="15"/>
       <c r="C94" s="14"/>
@@ -10419,7 +10430,7 @@
       <c r="CO94" s="14"/>
       <c r="CP94" s="14"/>
     </row>
-    <row r="95" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A95" s="5"/>
       <c r="B95" s="15"/>
       <c r="C95" s="14"/>
@@ -10515,7 +10526,7 @@
       <c r="CO95" s="14"/>
       <c r="CP95" s="14"/>
     </row>
-    <row r="96" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A96" s="5"/>
       <c r="B96" s="15"/>
       <c r="C96" s="14"/>
@@ -10611,7 +10622,7 @@
       <c r="CO96" s="14"/>
       <c r="CP96" s="14"/>
     </row>
-    <row r="97" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A97" s="5"/>
       <c r="B97" s="15"/>
       <c r="C97" s="14"/>
@@ -10707,7 +10718,7 @@
       <c r="CO97" s="14"/>
       <c r="CP97" s="14"/>
     </row>
-    <row r="98" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A98" s="5"/>
       <c r="B98" s="15"/>
       <c r="C98" s="14"/>
@@ -10803,7 +10814,7 @@
       <c r="CO98" s="14"/>
       <c r="CP98" s="14"/>
     </row>
-    <row r="99" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A99" s="5"/>
       <c r="B99" s="15"/>
       <c r="C99" s="14"/>
@@ -10899,7 +10910,7 @@
       <c r="CO99" s="14"/>
       <c r="CP99" s="14"/>
     </row>
-    <row r="100" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A100" s="5"/>
       <c r="B100" s="15"/>
       <c r="C100" s="14"/>
@@ -10995,7 +11006,7 @@
       <c r="CO100" s="14"/>
       <c r="CP100" s="14"/>
     </row>
-    <row r="101" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A101" s="5"/>
       <c r="B101" s="15"/>
       <c r="C101" s="14"/>
@@ -11091,7 +11102,7 @@
       <c r="CO101" s="14"/>
       <c r="CP101" s="14"/>
     </row>
-    <row r="102" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A102" s="5"/>
       <c r="B102" s="15"/>
       <c r="C102" s="14"/>
@@ -11187,7 +11198,7 @@
       <c r="CO102" s="14"/>
       <c r="CP102" s="14"/>
     </row>
-    <row r="103" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A103" s="5"/>
       <c r="B103" s="15"/>
       <c r="C103" s="14"/>
@@ -11283,7 +11294,7 @@
       <c r="CO103" s="14"/>
       <c r="CP103" s="14"/>
     </row>
-    <row r="104" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A104" s="5"/>
       <c r="B104" s="15"/>
       <c r="C104" s="14"/>
@@ -11379,7 +11390,7 @@
       <c r="CO104" s="14"/>
       <c r="CP104" s="14"/>
     </row>
-    <row r="105" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A105" s="5"/>
       <c r="B105" s="15"/>
       <c r="C105" s="14"/>
@@ -11475,7 +11486,7 @@
       <c r="CO105" s="14"/>
       <c r="CP105" s="14"/>
     </row>
-    <row r="106" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A106" s="5"/>
       <c r="B106" s="15"/>
       <c r="C106" s="14"/>
@@ -11571,7 +11582,7 @@
       <c r="CO106" s="14"/>
       <c r="CP106" s="14"/>
     </row>
-    <row r="107" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A107" s="5"/>
       <c r="B107" s="15"/>
       <c r="C107" s="14"/>
@@ -11667,7 +11678,7 @@
       <c r="CO107" s="14"/>
       <c r="CP107" s="14"/>
     </row>
-    <row r="108" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A108" s="5"/>
       <c r="B108" s="15"/>
       <c r="C108" s="14"/>
@@ -11763,7 +11774,7 @@
       <c r="CO108" s="14"/>
       <c r="CP108" s="14"/>
     </row>
-    <row r="109" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A109" s="5"/>
       <c r="B109" s="15"/>
       <c r="C109" s="14"/>
@@ -11859,7 +11870,7 @@
       <c r="CO109" s="14"/>
       <c r="CP109" s="14"/>
     </row>
-    <row r="110" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A110" s="5"/>
       <c r="B110" s="15"/>
       <c r="C110" s="14"/>
@@ -11955,7 +11966,7 @@
       <c r="CO110" s="14"/>
       <c r="CP110" s="14"/>
     </row>
-    <row r="111" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A111" s="5"/>
       <c r="B111" s="15"/>
       <c r="C111" s="14"/>
@@ -12051,7 +12062,7 @@
       <c r="CO111" s="14"/>
       <c r="CP111" s="14"/>
     </row>
-    <row r="112" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A112" s="5"/>
       <c r="B112" s="15"/>
       <c r="C112" s="14"/>
@@ -12147,7 +12158,7 @@
       <c r="CO112" s="14"/>
       <c r="CP112" s="14"/>
     </row>
-    <row r="113" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A113" s="5"/>
       <c r="B113" s="15"/>
       <c r="C113" s="14"/>
@@ -12243,7 +12254,7 @@
       <c r="CO113" s="14"/>
       <c r="CP113" s="14"/>
     </row>
-    <row r="114" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A114" s="5"/>
       <c r="B114" s="15"/>
       <c r="C114" s="14"/>
@@ -12339,7 +12350,7 @@
       <c r="CO114" s="14"/>
       <c r="CP114" s="14"/>
     </row>
-    <row r="115" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A115" s="5"/>
       <c r="B115" s="15"/>
       <c r="C115" s="14"/>
@@ -12435,7 +12446,7 @@
       <c r="CO115" s="14"/>
       <c r="CP115" s="14"/>
     </row>
-    <row r="116" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A116" s="5"/>
       <c r="B116" s="15"/>
       <c r="C116" s="14"/>
@@ -12531,7 +12542,7 @@
       <c r="CO116" s="14"/>
       <c r="CP116" s="14"/>
     </row>
-    <row r="117" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A117" s="5"/>
       <c r="B117" s="15"/>
       <c r="C117" s="14"/>
@@ -12627,7 +12638,7 @@
       <c r="CO117" s="14"/>
       <c r="CP117" s="14"/>
     </row>
-    <row r="118" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A118" s="5"/>
       <c r="B118" s="15"/>
       <c r="C118" s="14"/>
@@ -12723,7 +12734,7 @@
       <c r="CO118" s="14"/>
       <c r="CP118" s="14"/>
     </row>
-    <row r="119" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A119" s="5"/>
       <c r="B119" s="15"/>
       <c r="C119" s="14"/>
@@ -12819,7 +12830,7 @@
       <c r="CO119" s="14"/>
       <c r="CP119" s="14"/>
     </row>
-    <row r="120" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A120" s="5"/>
       <c r="B120" s="15"/>
       <c r="C120" s="14"/>
@@ -12915,7 +12926,7 @@
       <c r="CO120" s="14"/>
       <c r="CP120" s="14"/>
     </row>
-    <row r="121" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A121" s="5"/>
       <c r="B121" s="15"/>
       <c r="C121" s="14"/>
@@ -13011,7 +13022,7 @@
       <c r="CO121" s="14"/>
       <c r="CP121" s="14"/>
     </row>
-    <row r="122" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A122" s="5"/>
       <c r="B122" s="15"/>
       <c r="C122" s="14"/>
@@ -13107,7 +13118,7 @@
       <c r="CO122" s="14"/>
       <c r="CP122" s="14"/>
     </row>
-    <row r="123" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A123" s="5"/>
       <c r="B123" s="15"/>
       <c r="C123" s="14"/>
@@ -13203,7 +13214,7 @@
       <c r="CO123" s="14"/>
       <c r="CP123" s="14"/>
     </row>
-    <row r="124" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A124" s="5"/>
       <c r="B124" s="15"/>
       <c r="C124" s="14"/>
@@ -13299,7 +13310,7 @@
       <c r="CO124" s="14"/>
       <c r="CP124" s="14"/>
     </row>
-    <row r="125" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A125" s="5"/>
       <c r="B125" s="15"/>
       <c r="C125" s="14"/>
@@ -13395,7 +13406,7 @@
       <c r="CO125" s="14"/>
       <c r="CP125" s="14"/>
     </row>
-    <row r="126" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A126" s="5"/>
       <c r="B126" s="15"/>
       <c r="C126" s="14"/>
@@ -13491,7 +13502,7 @@
       <c r="CO126" s="14"/>
       <c r="CP126" s="14"/>
     </row>
-    <row r="127" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A127" s="5"/>
       <c r="B127" s="15"/>
       <c r="C127" s="14"/>
@@ -13587,7 +13598,7 @@
       <c r="CO127" s="14"/>
       <c r="CP127" s="14"/>
     </row>
-    <row r="128" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A128" s="5"/>
       <c r="B128" s="15"/>
       <c r="C128" s="14"/>
@@ -13683,7 +13694,7 @@
       <c r="CO128" s="14"/>
       <c r="CP128" s="14"/>
     </row>
-    <row r="129" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A129" s="5"/>
       <c r="B129" s="15"/>
       <c r="C129" s="14"/>
@@ -13779,7 +13790,7 @@
       <c r="CO129" s="14"/>
       <c r="CP129" s="14"/>
     </row>
-    <row r="130" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A130" s="5"/>
       <c r="B130" s="15"/>
       <c r="C130" s="14"/>
@@ -13875,7 +13886,7 @@
       <c r="CO130" s="14"/>
       <c r="CP130" s="14"/>
     </row>
-    <row r="131" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A131" s="5"/>
       <c r="B131" s="15"/>
       <c r="C131" s="14"/>
@@ -13971,7 +13982,7 @@
       <c r="CO131" s="14"/>
       <c r="CP131" s="14"/>
     </row>
-    <row r="132" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A132" s="5"/>
       <c r="B132" s="15"/>
       <c r="C132" s="14"/>
@@ -14067,7 +14078,7 @@
       <c r="CO132" s="14"/>
       <c r="CP132" s="14"/>
     </row>
-    <row r="133" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A133" s="5"/>
       <c r="B133" s="15"/>
       <c r="C133" s="14"/>
@@ -14163,7 +14174,7 @@
       <c r="CO133" s="14"/>
       <c r="CP133" s="14"/>
     </row>
-    <row r="134" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A134" s="5"/>
       <c r="B134" s="15"/>
       <c r="C134" s="14"/>
@@ -14259,7 +14270,7 @@
       <c r="CO134" s="14"/>
       <c r="CP134" s="14"/>
     </row>
-    <row r="135" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A135" s="5"/>
       <c r="B135" s="15"/>
       <c r="C135" s="14"/>
@@ -14355,7 +14366,7 @@
       <c r="CO135" s="14"/>
       <c r="CP135" s="14"/>
     </row>
-    <row r="136" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A136" s="5"/>
       <c r="B136" s="15"/>
       <c r="C136" s="14"/>
@@ -14451,7 +14462,7 @@
       <c r="CO136" s="14"/>
       <c r="CP136" s="14"/>
     </row>
-    <row r="137" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A137" s="5"/>
       <c r="B137" s="15"/>
       <c r="C137" s="14"/>
@@ -14547,7 +14558,7 @@
       <c r="CO137" s="14"/>
       <c r="CP137" s="14"/>
     </row>
-    <row r="138" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A138" s="5"/>
       <c r="B138" s="15"/>
       <c r="C138" s="14"/>
@@ -14643,7 +14654,7 @@
       <c r="CO138" s="14"/>
       <c r="CP138" s="14"/>
     </row>
-    <row r="139" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A139" s="5"/>
       <c r="B139" s="15"/>
       <c r="C139" s="14"/>
@@ -14739,7 +14750,7 @@
       <c r="CO139" s="14"/>
       <c r="CP139" s="14"/>
     </row>
-    <row r="140" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A140" s="5"/>
       <c r="B140" s="15"/>
       <c r="C140" s="14"/>
@@ -14835,7 +14846,7 @@
       <c r="CO140" s="14"/>
       <c r="CP140" s="14"/>
     </row>
-    <row r="141" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A141" s="5"/>
       <c r="B141" s="15"/>
       <c r="C141" s="14"/>
@@ -14931,7 +14942,7 @@
       <c r="CO141" s="14"/>
       <c r="CP141" s="14"/>
     </row>
-    <row r="142" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A142" s="5"/>
       <c r="B142" s="15"/>
       <c r="C142" s="14"/>
@@ -15027,7 +15038,7 @@
       <c r="CO142" s="14"/>
       <c r="CP142" s="14"/>
     </row>
-    <row r="143" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A143" s="5"/>
       <c r="B143" s="15"/>
       <c r="C143" s="14"/>
@@ -15123,7 +15134,7 @@
       <c r="CO143" s="14"/>
       <c r="CP143" s="14"/>
     </row>
-    <row r="144" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A144" s="5"/>
       <c r="B144" s="15"/>
       <c r="C144" s="14"/>
@@ -15219,7 +15230,7 @@
       <c r="CO144" s="14"/>
       <c r="CP144" s="14"/>
     </row>
-    <row r="145" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A145" s="5"/>
       <c r="B145" s="15"/>
       <c r="C145" s="14"/>
@@ -15315,7 +15326,7 @@
       <c r="CO145" s="14"/>
       <c r="CP145" s="14"/>
     </row>
-    <row r="146" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A146" s="5"/>
       <c r="B146" s="15"/>
       <c r="C146" s="14"/>
@@ -15411,7 +15422,7 @@
       <c r="CO146" s="14"/>
       <c r="CP146" s="14"/>
     </row>
-    <row r="147" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A147" s="5"/>
       <c r="B147" s="15"/>
       <c r="C147" s="14"/>
@@ -15507,7 +15518,7 @@
       <c r="CO147" s="14"/>
       <c r="CP147" s="14"/>
     </row>
-    <row r="148" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A148" s="5"/>
       <c r="B148" s="15"/>
       <c r="C148" s="14"/>
@@ -15603,7 +15614,7 @@
       <c r="CO148" s="14"/>
       <c r="CP148" s="14"/>
     </row>
-    <row r="149" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A149" s="5"/>
       <c r="B149" s="15"/>
       <c r="C149" s="14"/>
@@ -15699,7 +15710,7 @@
       <c r="CO149" s="14"/>
       <c r="CP149" s="14"/>
     </row>
-    <row r="150" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A150" s="5"/>
       <c r="B150" s="15"/>
       <c r="C150" s="14"/>
@@ -15795,7 +15806,7 @@
       <c r="CO150" s="14"/>
       <c r="CP150" s="14"/>
     </row>
-    <row r="151" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:94" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A151" s="5"/>
       <c r="B151" s="15"/>
       <c r="C151" s="14"/>

</xml_diff>